<commit_message>
[UPD] 12.0 sync from gitlab
</commit_message>
<xml_diff>
--- a/import_template_product_variant/tests/sample_template_without_variants.xlsx
+++ b/import_template_product_variant/tests/sample_template_without_variants.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t xml:space="preserve">product_tmpl_code</t>
   </si>
@@ -82,6 +82,9 @@
     <t xml:space="preserve">*TMPL*product_brand_id</t>
   </si>
   <si>
+    <t xml:space="preserve">route_ids</t>
+  </si>
+  <si>
     <t xml:space="preserve">PRODTMPL1TEST</t>
   </si>
   <si>
@@ -119,6 +122,9 @@
   </si>
   <si>
     <t xml:space="preserve">Brand 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make To Order</t>
   </si>
 </sst>
 </file>
@@ -210,23 +216,23 @@
     </xf>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T1048576"/>
-  <sheetFormatPr defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:U2"/>
+  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.89"/>
@@ -234,14 +240,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.28"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="17.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="69.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="15" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1023" min="18" style="0" width="8.91"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="1024" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -305,31 +310,34 @@
       <c r="T1" s="0" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="0" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="0" t="n">
         <v>4050119164021</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K2" s="0" t="n">
         <v>10.5</v>
@@ -338,36 +346,34 @@
         <v>15.99</v>
       </c>
       <c r="M2" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N2" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P2" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q2" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R2" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S2" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="T2" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="U2" s="0" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>